<commit_message>
added new request logic
</commit_message>
<xml_diff>
--- a/src/AutoTagSheet.xlsx
+++ b/src/AutoTagSheet.xlsx
@@ -8,15 +8,13 @@
   </bookViews>
   <sheets>
     <sheet sheetId="1" name="Vehicles" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Status Report" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Legend" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Column A</t>
   </si>
@@ -70,61 +68,13 @@
   </si>
   <si>
     <t>OD14T0649</t>
-  </si>
-  <si>
-    <t>STATUS LEGEND</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Text Color</t>
-  </si>
-  <si>
-    <t>Meaning</t>
-  </si>
-  <si>
-    <t>Tagged</t>
-  </si>
-  <si>
-    <t>Green</t>
-  </si>
-  <si>
-    <t>Record was successfully tagged</t>
-  </si>
-  <si>
-    <t>Already Tagged</t>
-  </si>
-  <si>
-    <t>Red</t>
-  </si>
-  <si>
-    <t>Record was already tagged, skipped</t>
-  </si>
-  <si>
-    <t>Failed</t>
-  </si>
-  <si>
-    <t>Orange</t>
-  </si>
-  <si>
-    <t>Record processing failed</t>
-  </si>
-  <si>
-    <t>Pending</t>
-  </si>
-  <si>
-    <t>Black</t>
-  </si>
-  <si>
-    <t>Record not yet processed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -144,40 +94,8 @@
       <sz val="11"/>
       <name val="Arial"/>
     </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFF0000"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF00B050"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFF9900"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF000000"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -189,18 +107,8 @@
         <fgColor rgb="FF1E293B"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF366092"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE7E6E6"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -238,26 +146,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -268,42 +161,52 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -652,166 +555,11 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A2:C6"/>
+  <conditionalFormatting sqref="A2:C6"/>
+  <conditionalFormatting sqref="A2:C6"/>
+  <conditionalFormatting sqref="A2:C6"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="3" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="40" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9"/>
-    </row>
-    <row r="3" spans="1:3" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>33</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
 </file>
</xml_diff>